<commit_message>
Fix definitions xlsx columns + add API fallback script
1. Match Matrixify's exact column names for definition imports:
   - "Owner Type" instead of "Owner"
   - "Pin" instead of "Pinned"
   - "Storefront Visibility" instead of "Visible to Storefront"
   - lowercase true/false
   - Added empty Validations column
   - Added empty ID column at the front

2. New create_definitions_via_api.py — Shopify GraphQL Admin API
   script that creates the kit_review metaobject + all 17 metafield
   definitions in one shot. Used as a fallback when Matrixify's
   definitions importer keeps misinterpreting the sheet as a values
   import. Idempotent: skips definitions that already exist.

https://claude.ai/code/session_01KsqRUKVeS9XsauvUkmk2pt
</commit_message>
<xml_diff>
--- a/shopify/matrixify/Sprout-Maker-Metafield-Definitions.xlsx
+++ b/shopify/matrixify/Sprout-Maker-Metafield-Definitions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -430,848 +430,892 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Command</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Owner Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Namespace</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Pinned</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Visible to Storefront</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Storefront Visibility</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Validations</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>activity_items</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Activity Items</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Hero activity row items. Each entry: "&lt;emoji&gt;|&lt;text&gt;". e.g. "⚡|Fresh sprouts in 2–3 days"</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>list.single_line_text_field</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>benefits_items</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Benefits Items</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Hero "Why this kit" 2x2 benefits. Each entry: "&lt;emoji&gt;|&lt;label&gt;". e.g. "🌱|Fresh sprouts in 2–3 days"</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>list.single_line_text_field</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>hero_trust_strip</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Hero Trust Strip</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Short trust items shown below the ATC button. e.g. Free Shipping / FSSAI Licensed</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>list.single_line_text_field</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>jar_capacity</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Jar Capacity</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Capacity label for the variant cards. "700ml" or "1000ml"</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>single_line_text_field</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>help_note</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Help Note</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Helper text shown beside the Jar Size Chart link in the variant block</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>multi_line_text_field</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>jar_size_chart_image</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Jar Size Chart Image</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Image displayed inside the Jar Size Chart modal</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>file_reference</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>companion_size_product</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Companion Size Product</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>The other capacity (700ml ↔ 1L) — drives the cross-capacity link below the variant block</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>product_reference</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>cross_sell_products</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Cross-sell Products</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Up to 3 products shown in the Pair It With section</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>list.product_reference</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>hero_benefits_icons</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Hero Benefits Icons (SVG)</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>Hero Benefits Icons</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>Custom SVG / image icons for the "Why this kit" 2x2 grid in the hero. List in the same order as benefits_items. Overrides the emoji prefix.</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>list.file_reference</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>benefits_icons</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Benefits Icons (SVG)</t>
-        </is>
-      </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>Benefits Icons</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>Custom SVG / image icons for the "Quick Benefits" 3-card section. List in the same order as benefit blocks.</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>list.file_reference</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>comparison_left_image</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Comparison Left Image</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Image for the LEFT side of the comparison section (cloth method). Overrides the section setting.</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>file_reference</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>comparison_right_image</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Comparison Right Image</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Image for the RIGHT side of the comparison section (sprout maker). Overrides the section setting.</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>file_reference</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>box_image</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Box / Kit Image</t>
-        </is>
-      </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>Box Image</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
           <t>Image for the What's in the Box section. Overrides the section setting.</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>file_reference</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>how_to_make_video</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>How to Make Video</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Demo video for the How to Make section. Overrides the section setting.</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>file_reference</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>MERGE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>featured_reviews</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Featured Reviews</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>List of kit_review metaobjects shown in the UGC Reviews section. Overrides the manual review blocks.</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>list.metaobject_reference</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
+          <t>MERGE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>Product Variant</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>custom</t>
-        </is>
-      </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>best_for</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Best For</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Per-variant audience copy under the BEST FOR label inside each pack card</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>single_line_text_field</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>MERGE</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
+          <t>MERGE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>Product Variant</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>custom</t>
-        </is>
-      </c>
       <c r="D18" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>tag</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Variant Tag</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Optional badge above each variant card. e.g. TOP SELLER, BEST VALUE</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>single_line_text_field</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>